<commit_message>
final production ready 🚀
</commit_message>
<xml_diff>
--- a/data/menu.xlsx
+++ b/data/menu.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="22188" windowHeight="8280"/>
+    <workbookView windowWidth="22188" windowHeight="9000"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="408" uniqueCount="175">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="423" uniqueCount="181">
   <si>
     <t>Name</t>
   </si>
@@ -122,7 +122,7 @@
     <t>Chilly Paneer (5 pcs) + Veg Fried Rice + 2 Lacha Paratha</t>
   </si>
   <si>
-    <t xml:space="preserve"> Mega Combos</t>
+    <t>Littiwale Mega Feast</t>
   </si>
   <si>
     <t>Littiwale Mega Feast - Chilly Chicken Veg Fried Rice Lacha Paratha</t>
@@ -149,7 +149,7 @@
     <t>Chilly Paneer (4 pcs) + Lacha Paratha</t>
   </si>
   <si>
-    <t xml:space="preserve"> Mini Combos</t>
+    <t>Littiwale Meal for One</t>
   </si>
   <si>
     <t>Meals for one - Veg Noodles Paneer Chilly</t>
@@ -239,7 +239,7 @@
     <t>Veg Noodles (Half)</t>
   </si>
   <si>
-    <t xml:space="preserve"> Noodles  Rice</t>
+    <t xml:space="preserve"> Noodles/Rice</t>
   </si>
   <si>
     <t>Veg Noodles (Full)</t>
@@ -257,10 +257,10 @@
     <t>Chicken Noodles (Full)</t>
   </si>
   <si>
-    <t>Mix  Veg Noodles (Half)</t>
-  </si>
-  <si>
-    <t>Mix  Veg Noodles (Full)</t>
+    <t>Mix Veg Noodles (Half)</t>
+  </si>
+  <si>
+    <t>Mix Veg Noodles (Full)</t>
   </si>
   <si>
     <t>Mix Non Veg Noodles (Half)</t>
@@ -344,7 +344,7 @@
     <t>1 pc</t>
   </si>
   <si>
-    <t xml:space="preserve"> Parathas  Naan</t>
+    <t>Breads</t>
   </si>
   <si>
     <t>Butter Naan</t>
@@ -377,7 +377,7 @@
     <t>Veg Pizza</t>
   </si>
   <si>
-    <t xml:space="preserve"> Pizzas</t>
+    <t xml:space="preserve"> Pizza</t>
   </si>
   <si>
     <t>Corn Pizza</t>
@@ -407,7 +407,7 @@
     <t>Veg Maggie (Half)</t>
   </si>
   <si>
-    <t xml:space="preserve"> Maggi  Snacks</t>
+    <t xml:space="preserve"> Maggi</t>
   </si>
   <si>
     <t>Veg Maggie (Full)</t>
@@ -446,10 +446,10 @@
     <t>Paneer Butter Masala (Full)</t>
   </si>
   <si>
-    <t>Panner Masala (Half)</t>
-  </si>
-  <si>
-    <t>Panner Masala (Full)</t>
+    <t>Paneer Masala (Half)</t>
+  </si>
+  <si>
+    <t>Paneer Masala (Full)</t>
   </si>
   <si>
     <t>Palak Paneer (Half)</t>
@@ -552,6 +552,24 @@
   </si>
   <si>
     <t>Roti(5pc) or (Rice+Dal)+Muttton Curry (4 pcs)+ 1 type of Bhujia+Papad</t>
+  </si>
+  <si>
+    <t>Masterchef Special Thecha Chowmein (Half)</t>
+  </si>
+  <si>
+    <t>Masterchef Special Thecha Chowmein (Full)</t>
+  </si>
+  <si>
+    <t>Rajma Chawal</t>
+  </si>
+  <si>
+    <t>Littiwale Rice Bowl Combos</t>
+  </si>
+  <si>
+    <t>Chole Chawal</t>
+  </si>
+  <si>
+    <t>Kadhi Chawal</t>
   </si>
 </sst>
 </file>
@@ -1539,7 +1557,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:G117"/>
+  <dimension ref="A1:G122"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="14.4" outlineLevelCol="6"/>
   <cols>
     <col min="1" max="1" width="59.7777777777778" customWidth="1"/>
@@ -3704,6 +3722,91 @@
         <v>164</v>
       </c>
     </row>
+    <row r="118" spans="1:6">
+      <c r="A118" t="s">
+        <v>175</v>
+      </c>
+      <c r="C118">
+        <v>79</v>
+      </c>
+      <c r="D118" t="s">
+        <v>8</v>
+      </c>
+      <c r="E118" t="s">
+        <v>9</v>
+      </c>
+      <c r="F118" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6">
+      <c r="A119" t="s">
+        <v>176</v>
+      </c>
+      <c r="C119">
+        <v>149</v>
+      </c>
+      <c r="D119" t="s">
+        <v>8</v>
+      </c>
+      <c r="E119" t="s">
+        <v>9</v>
+      </c>
+      <c r="F119" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6">
+      <c r="A120" t="s">
+        <v>177</v>
+      </c>
+      <c r="C120">
+        <v>79</v>
+      </c>
+      <c r="D120" t="s">
+        <v>178</v>
+      </c>
+      <c r="E120" t="s">
+        <v>9</v>
+      </c>
+      <c r="F120" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6">
+      <c r="A121" t="s">
+        <v>179</v>
+      </c>
+      <c r="C121">
+        <v>79</v>
+      </c>
+      <c r="D121" t="s">
+        <v>178</v>
+      </c>
+      <c r="E121" t="s">
+        <v>9</v>
+      </c>
+      <c r="F121" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6">
+      <c r="A122" t="s">
+        <v>180</v>
+      </c>
+      <c r="C122">
+        <v>79</v>
+      </c>
+      <c r="D122" t="s">
+        <v>178</v>
+      </c>
+      <c r="E122" t="s">
+        <v>9</v>
+      </c>
+      <c r="F122" t="b">
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <headerFooter/>

</xml_diff>